<commit_message>
add il and ita
</commit_message>
<xml_diff>
--- a/8il/assign/23il-students.xlsx
+++ b/8il/assign/23il-students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Freeman/Documents/college/slides/8il/assign/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE5E02DA-A40F-4E4C-8957-640A112E1462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C919575-6D9C-704C-9BE4-E98737DE450F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15180" yWindow="7700" windowWidth="27640" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>